<commit_message>
Update services & planning file
</commit_message>
<xml_diff>
--- a/data/planning/ASIN Planning file - Feb 2026.xlsx
+++ b/data/planning/ASIN Planning file - Feb 2026.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\Week 5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\FAstAPIc\data\planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F8CE87F-8D1F-4685-AAE4-99816ED13064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF5061D-9D4B-494B-9D38-826D0C5DD5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B42A6E69-4368-4E62-9729-C9D7959FE44A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{B42A6E69-4368-4E62-9729-C9D7959FE44A}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
     <sheet name="Category" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Main!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Main!$A$1:$H$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="171">
   <si>
     <t>Brand</t>
   </si>
@@ -413,6 +413,144 @@
   </si>
   <si>
     <t>Feb Goal</t>
+  </si>
+  <si>
+    <t>productname</t>
+  </si>
+  <si>
+    <t>NexLev Smart Air Purifier</t>
+  </si>
+  <si>
+    <t>Nexlev Electric Toothbrush</t>
+  </si>
+  <si>
+    <t>NexLev Professional Air Purifier for 650 sq ft Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Mattress, Sofa &amp; Carpet Vacuum Cleaner </t>
+  </si>
+  <si>
+    <t>NexLev Mattress, Sofa, Carpet &amp; Car Seat Vacuum Cleaner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Steam Cleaner </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nexlev SWIPE Steam Cleaner </t>
+  </si>
+  <si>
+    <t>NexLev 10 in 1 Steam Cleaner &amp; Mop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Steam Mop </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev 2 in 1 Handheld &amp; Stick Vacuum Cleaner </t>
+  </si>
+  <si>
+    <t>NexLev Cordless Wet &amp; Dry Vacuum Cleaner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Handheld Garment Steamer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Foldable Garment Steamer for Home &amp; Travel </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Portable Cordless Lint Remover </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Rechargeable Lint Remover </t>
+  </si>
+  <si>
+    <t>Nexlev Portable Sewing Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Stand Mixer </t>
+  </si>
+  <si>
+    <t>Nexlev MultiPurpose Electric Food Kettle</t>
+  </si>
+  <si>
+    <t>Nexlev Multi Purpose Electric Food Kettle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Portable Blender for Smoothies Milkshakes Crushing Ice Juices </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Mini Electric Chopper </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev 1500W Electric Water Kettle </t>
+  </si>
+  <si>
+    <t>NexLev Portable Tyre Inflator for Car, Bike, Cycle</t>
+  </si>
+  <si>
+    <t>NexLev Steamer For Cold &amp; Cough</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Blackhead &amp; Whitehead Remover Tool </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Foot Callus Remover </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nexlev Skin Scrubber </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nexlev Skin Lift Device </t>
+  </si>
+  <si>
+    <t>nexlev Ionic 3 In 1 Hot Air Brush</t>
+  </si>
+  <si>
+    <t>nexlev Ionic Volumizer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Ionic Hot Air Brush </t>
+  </si>
+  <si>
+    <t>NexLev IONIC Volumizer + Straightening Brush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Ionic Cordless Hair Straightener Brush </t>
+  </si>
+  <si>
+    <t>NexLev Ionic Hair Straightener Brush for Woman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev LED Phototherapy comb </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nexlev Just Style Pro Hair Dryer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev LED Therapy Oil Applicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Calf Massager </t>
+  </si>
+  <si>
+    <t>NexLev Cordless Electric Heating Pad</t>
+  </si>
+  <si>
+    <t>NexLev Calf Massager Pro</t>
+  </si>
+  <si>
+    <t>NexLev Intimate Trimmer for Men</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev All in One Body Trimmer for Men </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev 6-in-1 trimmer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NexLev Smart Electric Toothbrush for Adults </t>
+  </si>
+  <si>
+    <t>Nexlev Rechargeable Electric Toothbrush</t>
   </si>
 </sst>
 </file>
@@ -836,1031 +974,1192 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4372B9CE-A816-4945-A3DD-FAB6EC08913C}">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.109375" style="2"/>
+    <col min="2" max="2" width="58.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="9">
+      <c r="E2" s="9">
         <v>542238</v>
       </c>
-      <c r="E2" s="9">
+      <c r="F2" s="9">
         <v>19366</v>
       </c>
-      <c r="F2" s="9"/>
       <c r="G2" s="9"/>
-    </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="9">
+      <c r="E3" s="9">
         <v>237119</v>
       </c>
-      <c r="E3" s="9">
+      <c r="F3" s="9">
         <v>8469</v>
       </c>
-      <c r="F3" s="9"/>
       <c r="G3" s="9"/>
-    </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H3" s="9"/>
+    </row>
+    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="9">
+      <c r="E4" s="9">
         <v>687899</v>
       </c>
-      <c r="E4" s="9">
+      <c r="F4" s="9">
         <v>24568</v>
       </c>
-      <c r="F4" s="9"/>
       <c r="G4" s="9"/>
-    </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="9">
+      <c r="E5" s="9">
         <v>475284</v>
       </c>
-      <c r="E5" s="9">
+      <c r="F5" s="9">
         <v>16975</v>
       </c>
-      <c r="F5" s="9"/>
       <c r="G5" s="9"/>
-    </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H5" s="9"/>
+    </row>
+    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="9">
+      <c r="E6" s="9">
         <v>614195</v>
       </c>
-      <c r="E6" s="9">
+      <c r="F6" s="9">
         <v>21936</v>
       </c>
-      <c r="F6" s="9"/>
       <c r="G6" s="9"/>
-    </row>
-    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H6" s="9"/>
+    </row>
+    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D7" s="9">
+      <c r="E7" s="9">
         <v>889577</v>
       </c>
-      <c r="E7" s="9">
+      <c r="F7" s="9">
         <v>31771</v>
       </c>
-      <c r="F7" s="9"/>
       <c r="G7" s="9"/>
-    </row>
-    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H7" s="9"/>
+    </row>
+    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="9">
+      <c r="E8" s="9">
         <v>244034</v>
       </c>
-      <c r="E8" s="9">
+      <c r="F8" s="9">
         <v>8716</v>
       </c>
-      <c r="F8" s="9"/>
       <c r="G8" s="9"/>
-    </row>
-    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="9">
+      <c r="E9" s="9">
         <v>1016780</v>
       </c>
-      <c r="E9" s="9">
+      <c r="F9" s="9">
         <v>36314</v>
       </c>
-      <c r="F9" s="9"/>
       <c r="G9" s="9"/>
-    </row>
-    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H9" s="9"/>
+    </row>
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D10" s="9">
+      <c r="E10" s="9">
         <v>152505</v>
       </c>
-      <c r="E10" s="9">
+      <c r="F10" s="9">
         <v>5447</v>
       </c>
-      <c r="F10" s="9"/>
       <c r="G10" s="9"/>
-    </row>
-    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H10" s="9"/>
+    </row>
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="9">
+      <c r="E11" s="9">
         <v>355763</v>
       </c>
-      <c r="E11" s="9">
+      <c r="F11" s="9">
         <v>12706</v>
       </c>
-      <c r="F11" s="9"/>
       <c r="G11" s="9"/>
-    </row>
-    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H11" s="9"/>
+    </row>
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="D12" s="9">
+      <c r="E12" s="9">
         <v>97416</v>
       </c>
-      <c r="E12" s="9">
+      <c r="F12" s="9">
         <v>3480</v>
       </c>
-      <c r="F12" s="9"/>
       <c r="G12" s="9"/>
-    </row>
-    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="9"/>
+    </row>
+    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="9">
+      <c r="E13" s="9">
         <v>465890</v>
       </c>
-      <c r="E13" s="9">
+      <c r="F13" s="9">
         <v>16639</v>
       </c>
-      <c r="F13" s="9"/>
       <c r="G13" s="9"/>
-    </row>
-    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H13" s="9"/>
+    </row>
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="9">
+      <c r="E14" s="9">
         <v>235043</v>
       </c>
-      <c r="E14" s="9">
+      <c r="F14" s="9">
         <v>8395</v>
       </c>
-      <c r="F14" s="9"/>
       <c r="G14" s="9"/>
-    </row>
-    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H14" s="9"/>
+    </row>
+    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="9">
+      <c r="E15" s="9">
         <v>128475</v>
       </c>
-      <c r="E15" s="9">
+      <c r="F15" s="9">
         <v>4589</v>
       </c>
-      <c r="F15" s="9"/>
       <c r="G15" s="9"/>
-    </row>
-    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H15" s="9"/>
+    </row>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="9">
+      <c r="E16" s="9">
         <v>190551</v>
       </c>
-      <c r="E16" s="9">
+      <c r="F16" s="9">
         <v>6806</v>
       </c>
-      <c r="F16" s="9"/>
       <c r="G16" s="9"/>
-    </row>
-    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H16" s="9"/>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D17" s="9">
+      <c r="E17" s="9">
         <v>38094</v>
       </c>
-      <c r="E17" s="9">
+      <c r="F17" s="9">
         <v>1361</v>
       </c>
-      <c r="F17" s="9"/>
       <c r="G17" s="9"/>
-    </row>
-    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="D18" s="9">
+      <c r="E18" s="9">
         <v>167645</v>
       </c>
-      <c r="E18" s="9">
+      <c r="F18" s="9">
         <v>5988</v>
       </c>
-      <c r="F18" s="9"/>
       <c r="G18" s="9"/>
-    </row>
-    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D19" s="9">
+      <c r="E19" s="9">
         <v>565157</v>
       </c>
-      <c r="E19" s="9">
+      <c r="F19" s="9">
         <v>20185</v>
       </c>
-      <c r="F19" s="9"/>
       <c r="G19" s="9"/>
-    </row>
-    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H19" s="9"/>
+    </row>
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="9">
+      <c r="E20" s="9">
         <v>169386</v>
       </c>
-      <c r="E20" s="9">
+      <c r="F20" s="9">
         <v>6050</v>
       </c>
-      <c r="F20" s="9"/>
       <c r="G20" s="9"/>
-    </row>
-    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H20" s="9"/>
+    </row>
+    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D21" s="9">
+      <c r="E21" s="9">
         <v>148221</v>
       </c>
-      <c r="E21" s="9">
+      <c r="F21" s="9">
         <v>5294</v>
       </c>
-      <c r="F21" s="9"/>
       <c r="G21" s="9"/>
-    </row>
-    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H21" s="9"/>
+    </row>
+    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="D22" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D22" s="9">
+      <c r="E22" s="9">
         <v>149085</v>
       </c>
-      <c r="E22" s="9">
+      <c r="F22" s="9">
         <v>5325</v>
       </c>
-      <c r="F22" s="9"/>
       <c r="G22" s="9"/>
-    </row>
-    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="D23" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D23" s="9">
+      <c r="E23" s="9">
         <v>40611</v>
       </c>
-      <c r="E23" s="9">
+      <c r="F23" s="9">
         <v>1451</v>
       </c>
-      <c r="F23" s="9"/>
       <c r="G23" s="9"/>
-    </row>
-    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D24" s="9">
+      <c r="E24" s="9">
         <v>110000</v>
       </c>
-      <c r="E24" s="9">
+      <c r="F24" s="9">
         <v>3929</v>
       </c>
-      <c r="F24" s="9"/>
       <c r="G24" s="9"/>
-    </row>
-    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H24" s="9"/>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C25" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D25" s="9">
+      <c r="E25" s="9">
         <v>63517</v>
       </c>
-      <c r="E25" s="9">
+      <c r="F25" s="9">
         <v>2269</v>
       </c>
-      <c r="F25" s="9"/>
       <c r="G25" s="9"/>
-    </row>
-    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H25" s="9"/>
+    </row>
+    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="D26" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D26" s="9">
+      <c r="E26" s="9">
         <v>76229</v>
       </c>
-      <c r="E26" s="9">
+      <c r="F26" s="9">
         <v>2723</v>
       </c>
-      <c r="F26" s="9"/>
       <c r="G26" s="9"/>
-    </row>
-    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H26" s="9"/>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="C27" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="D27" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="9">
+      <c r="E27" s="9">
         <v>67755</v>
       </c>
-      <c r="E27" s="9">
+      <c r="F27" s="9">
         <v>2420</v>
       </c>
-      <c r="F27" s="9"/>
       <c r="G27" s="9"/>
-    </row>
-    <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H27" s="9"/>
+    </row>
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="D28" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D28" s="9">
+      <c r="E28" s="9">
         <v>29619</v>
       </c>
-      <c r="E28" s="9">
+      <c r="F28" s="9">
         <v>1058</v>
       </c>
-      <c r="F28" s="9"/>
       <c r="G28" s="9"/>
-    </row>
-    <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H28" s="9"/>
+    </row>
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="C29" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D29" s="9">
+      <c r="E29" s="9">
         <v>57594</v>
       </c>
-      <c r="E29" s="9">
+      <c r="F29" s="9">
         <v>2057</v>
       </c>
-      <c r="F29" s="9"/>
       <c r="G29" s="9"/>
-    </row>
-    <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H29" s="9"/>
+    </row>
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="D30" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D30" s="9">
+      <c r="E30" s="9">
         <v>63517</v>
       </c>
-      <c r="E30" s="9">
+      <c r="F30" s="9">
         <v>2269</v>
       </c>
-      <c r="F30" s="9"/>
       <c r="G30" s="9"/>
-    </row>
-    <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H30" s="9"/>
+    </row>
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="D31" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D31" s="9">
+      <c r="E31" s="9">
         <v>711526</v>
       </c>
-      <c r="E31" s="9">
+      <c r="F31" s="9">
         <v>25412</v>
       </c>
-      <c r="F31" s="9"/>
       <c r="G31" s="9"/>
-    </row>
-    <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H31" s="9"/>
+    </row>
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="C32" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="D32" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="D32" s="9">
+      <c r="E32" s="9">
         <v>158793</v>
       </c>
-      <c r="E32" s="9">
+      <c r="F32" s="9">
         <v>5672</v>
       </c>
-      <c r="F32" s="9"/>
       <c r="G32" s="9"/>
-    </row>
-    <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H32" s="9"/>
+    </row>
+    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="D33" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D33" s="9">
+      <c r="E33" s="9">
         <v>118560</v>
       </c>
-      <c r="E33" s="9">
+      <c r="F33" s="9">
         <v>4235</v>
       </c>
-      <c r="F33" s="9"/>
       <c r="G33" s="9"/>
-    </row>
-    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H33" s="9"/>
+    </row>
+    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C34" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="D34" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D34" s="9">
+      <c r="E34" s="9">
         <v>97416</v>
       </c>
-      <c r="E34" s="9">
+      <c r="F34" s="9">
         <v>3480</v>
       </c>
-      <c r="F34" s="9"/>
       <c r="G34" s="9"/>
-    </row>
-    <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H34" s="9"/>
+    </row>
+    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C35" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="D35" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D35" s="9">
+      <c r="E35" s="9">
         <v>311314</v>
       </c>
-      <c r="E35" s="9">
+      <c r="F35" s="9">
         <v>11119</v>
       </c>
-      <c r="F35" s="9"/>
       <c r="G35" s="9"/>
-    </row>
-    <row r="36" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H35" s="9"/>
+    </row>
+    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="D36" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D36" s="9">
+      <c r="E36" s="9">
         <v>160933</v>
       </c>
-      <c r="E36" s="9">
+      <c r="F36" s="9">
         <v>5748</v>
       </c>
-      <c r="F36" s="9"/>
       <c r="G36" s="9"/>
-    </row>
-    <row r="37" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H36" s="9"/>
+    </row>
+    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="C37" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="D37" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D37" s="9">
+      <c r="E37" s="9">
         <v>254111</v>
       </c>
-      <c r="E37" s="9">
+      <c r="F37" s="9">
         <v>9076</v>
       </c>
-      <c r="F37" s="9"/>
       <c r="G37" s="9"/>
-    </row>
-    <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H37" s="9"/>
+    </row>
+    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C38" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="D38" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D38" s="9">
+      <c r="E38" s="9">
         <v>71556</v>
       </c>
-      <c r="E38" s="9">
+      <c r="F38" s="9">
         <v>2556</v>
       </c>
-      <c r="F38" s="9"/>
       <c r="G38" s="9"/>
-    </row>
-    <row r="39" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H38" s="9"/>
+    </row>
+    <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="C39" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="D39" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="9">
+      <c r="E39" s="9">
         <v>125734</v>
       </c>
-      <c r="E39" s="9">
+      <c r="F39" s="9">
         <v>4491</v>
       </c>
-      <c r="F39" s="9"/>
       <c r="G39" s="9"/>
-    </row>
-    <row r="40" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H39" s="9"/>
+    </row>
+    <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C40" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="D40" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D40" s="9">
+      <c r="E40" s="9">
         <v>379526</v>
       </c>
-      <c r="E40" s="9">
+      <c r="F40" s="9">
         <v>13555</v>
       </c>
-      <c r="F40" s="9"/>
       <c r="G40" s="9"/>
-    </row>
-    <row r="41" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H40" s="9"/>
+    </row>
+    <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="D41" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D41" s="9">
+      <c r="E41" s="9">
         <v>66051</v>
       </c>
-      <c r="E41" s="9">
+      <c r="F41" s="9">
         <v>2359</v>
       </c>
-      <c r="F41" s="9"/>
       <c r="G41" s="9"/>
-    </row>
-    <row r="42" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H41" s="9"/>
+    </row>
+    <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="D42" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D42" s="9">
+      <c r="E42" s="9">
         <v>71136</v>
       </c>
-      <c r="E42" s="9">
+      <c r="F42" s="9">
         <v>2541</v>
       </c>
-      <c r="F42" s="9"/>
       <c r="G42" s="9"/>
-    </row>
-    <row r="43" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H42" s="9"/>
+    </row>
+    <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="C43" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="D43" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D43" s="9">
+      <c r="E43" s="9">
         <v>25420</v>
       </c>
-      <c r="E43" s="9">
+      <c r="F43" s="9">
         <v>908</v>
       </c>
-      <c r="F43" s="9"/>
       <c r="G43" s="9"/>
-    </row>
-    <row r="44" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H43" s="9"/>
+    </row>
+    <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="D44" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D44" s="9">
+      <c r="E44" s="9">
         <v>84729</v>
       </c>
-      <c r="E44" s="9">
+      <c r="F44" s="9">
         <v>3027</v>
       </c>
-      <c r="F44" s="9"/>
       <c r="G44" s="9"/>
-    </row>
-    <row r="45" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H44" s="9"/>
+    </row>
+    <row r="45" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="C45" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="D45" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D45" s="9">
+      <c r="E45" s="9">
         <v>88899</v>
       </c>
-      <c r="E45" s="9">
+      <c r="F45" s="9">
         <v>3175</v>
       </c>
-      <c r="F45" s="9"/>
       <c r="G45" s="9"/>
-    </row>
-    <row r="46" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H45" s="9"/>
+    </row>
+    <row r="46" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="B46" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C46" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="D46" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D46" s="9">
+      <c r="E46" s="9">
         <v>59589</v>
       </c>
-      <c r="E46" s="9">
+      <c r="F46" s="9">
         <v>2129</v>
       </c>
-      <c r="F46" s="9"/>
       <c r="G46" s="9"/>
-    </row>
-    <row r="47" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H46" s="9"/>
+    </row>
+    <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="C47" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="D47" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D47" s="9">
+      <c r="E47" s="9">
         <v>101611</v>
       </c>
-      <c r="E47" s="9">
+      <c r="F47" s="9">
         <v>3629</v>
       </c>
-      <c r="F47" s="9"/>
       <c r="G47" s="9"/>
-    </row>
-    <row r="48" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H47" s="9"/>
+    </row>
+    <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B48" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C48" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="D48" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D48" s="9">
+      <c r="E48" s="9">
         <v>50678</v>
       </c>
-      <c r="E48" s="9">
+      <c r="F48" s="9">
         <v>1810</v>
       </c>
-      <c r="F48" s="9"/>
       <c r="G48" s="9"/>
-    </row>
-    <row r="49" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H48" s="9"/>
+    </row>
+    <row r="49" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="D49" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D49" s="9">
+      <c r="E49" s="9">
         <v>25339</v>
       </c>
-      <c r="E49" s="9">
+      <c r="F49" s="9">
         <v>905</v>
       </c>
-      <c r="F49" s="9"/>
       <c r="G49" s="9"/>
-    </row>
-    <row r="50" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H49" s="9"/>
+    </row>
+    <row r="50" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C50" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="D50" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D50" s="9">
+      <c r="E50" s="9">
         <v>38085</v>
       </c>
-      <c r="E50" s="9">
+      <c r="F50" s="9">
         <v>1361</v>
       </c>
-      <c r="F50" s="9"/>
       <c r="G50" s="9"/>
-    </row>
-    <row r="51" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H50" s="9"/>
+    </row>
+    <row r="51" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B51" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C51" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="D51" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D51" s="9">
+      <c r="E51" s="9">
         <v>95212</v>
       </c>
-      <c r="E51" s="9">
+      <c r="F51" s="9">
         <v>3401</v>
       </c>
-      <c r="F51" s="9"/>
       <c r="G51" s="9"/>
-    </row>
-    <row r="52" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H51" s="9"/>
+    </row>
+    <row r="52" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B52" s="8" t="s">
+      <c r="B52" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C52" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C52" s="7" t="s">
+      <c r="D52" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D52" s="9">
+      <c r="E52" s="9">
         <v>16928</v>
       </c>
-      <c r="E52" s="9">
+      <c r="F52" s="9">
         <v>605</v>
       </c>
-      <c r="F52" s="9"/>
       <c r="G52" s="9"/>
-    </row>
-    <row r="53" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H52" s="9"/>
+    </row>
+    <row r="53" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C53" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C53" s="7" t="s">
+      <c r="D53" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="D53" s="9">
+      <c r="E53" s="9">
         <v>33856</v>
       </c>
-      <c r="E53" s="9">
+      <c r="F53" s="9">
         <v>1210</v>
       </c>
-      <c r="F53" s="9"/>
       <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H53" xr:uid="{4372B9CE-A816-4945-A3DD-FAB6EC08913C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>